<commit_message>
Stage 5: one-command pipeline replaces Dataiku (decision 31); improvements 7 and 10 done
</commit_message>
<xml_diff>
--- a/tableau/data/dashboard_data.xlsx
+++ b/tableau/data/dashboard_data.xlsx
@@ -489,11 +489,11 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>2</v>
+        <v>21</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -1685,7 +1685,7 @@
         <v>374600.83</v>
       </c>
       <c r="M3" t="n">
-        <v>11294964209.24</v>
+        <v>11294964209.23</v>
       </c>
     </row>
     <row r="4">

</xml_diff>